<commit_message>
Changes July 12 2024
</commit_message>
<xml_diff>
--- a/TestData/LV_T2276_T2277_EventExpenseEmailNotificationsRejectApproveRequestAsFirstLevelApprover.xlsx
+++ b/TestData/LV_T2276_T2277_EventExpenseEmailNotificationsRejectApproveRequestAsFirstLevelApprover.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\vkumar0427\source\repos\SF_Automation\TestData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8BF914B5-DCE9-45FE-AE30-FD6DA224A638}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F6D1FBA4-C33A-4E30-81EA-67D250A758BF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Users" sheetId="2" r:id="rId1"/>
@@ -510,19 +510,19 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:B3"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="14.28515625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="15.7109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="14.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="15.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>21</v>
       </c>
       <c r="B1" s="1"/>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>44</v>
       </c>
@@ -530,7 +530,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>44</v>
       </c>
@@ -544,17 +544,17 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{209E491E-EAF6-4396-A065-2D97079F795A}">
   <dimension ref="A1:A2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="10.28515625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="10.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>41</v>
       </c>
@@ -567,14 +567,17 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BC80C046-0B4F-4B58-AB08-7498887711A4}">
   <dimension ref="A1:A2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="19.77734375" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>43</v>
       </c>
@@ -587,27 +590,27 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:Q3"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="5.28515625" customWidth="1"/>
-    <col min="2" max="2" width="18.42578125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="14.28515625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="14.42578125" customWidth="1"/>
-    <col min="5" max="5" width="11.7109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="5.33203125" customWidth="1"/>
+    <col min="2" max="2" width="18.44140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="14.33203125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="14.44140625" customWidth="1"/>
+    <col min="5" max="5" width="11.6640625" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="21" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="7" customWidth="1"/>
-    <col min="8" max="8" width="22.7109375" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="10.28515625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="17.7109375" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="15.5703125" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="9.42578125" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="13.42578125" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="19.42578125" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="13.7109375" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="13.42578125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="22.6640625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="10.33203125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="17.6640625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="15.5546875" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="9.44140625" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="13.44140625" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="19.44140625" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="13.6640625" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="13.44140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -660,7 +663,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="2" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>24</v>
       </c>
@@ -713,7 +716,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="3" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>24</v>
       </c>
@@ -775,13 +778,13 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:F22"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="19.140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19.109375" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="14" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>29</v>
       </c>
@@ -789,7 +792,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" s="3" t="s">
         <v>34</v>
       </c>
@@ -797,7 +800,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3" s="3" t="s">
         <v>36</v>
       </c>
@@ -805,7 +808,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="22" spans="6:6" x14ac:dyDescent="0.25">
+    <row r="22" spans="6:6" x14ac:dyDescent="0.3">
       <c r="F22" t="s">
         <v>31</v>
       </c>
@@ -824,13 +827,13 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:B3"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="19.28515625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19.33203125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="14" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>29</v>
       </c>
@@ -838,7 +841,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" s="3" t="s">
         <v>34</v>
       </c>
@@ -846,7 +849,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3" s="3" t="s">
         <v>36</v>
       </c>

</xml_diff>

<commit_message>
LV_TMTT0012113 Changes July 19 2024
</commit_message>
<xml_diff>
--- a/TestData/LV_T2276_T2277_EventExpenseEmailNotificationsRejectApproveRequestAsFirstLevelApprover.xlsx
+++ b/TestData/LV_T2276_T2277_EventExpenseEmailNotificationsRejectApproveRequestAsFirstLevelApprover.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\vkumar0427\source\repos\SF_Automation\TestData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F6D1FBA4-C33A-4E30-81EA-67D250A758BF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CB1AC694-BF59-4BFA-A599-FBD66920CFB1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Users" sheetId="2" r:id="rId1"/>

</xml_diff>

<commit_message>
PRJ0094584-Add New Field to CM Opp/Eng Counterparty Page, Aug 13 2025
</commit_message>
<xml_diff>
--- a/TestData/LV_T2276_T2277_EventExpenseEmailNotificationsRejectApproveRequestAsFirstLevelApprover.xlsx
+++ b/TestData/LV_T2276_T2277_EventExpenseEmailNotificationsRejectApproveRequestAsFirstLevelApprover.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28623"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29029"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\vkumar0427\source\repos\SF_Automation\TestData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7BB3176C-D7FE-41F6-B93F-BDBBD47D972C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{313C0CC8-47FB-446E-8110-7617FE2D6B53}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-23148" yWindow="708" windowWidth="23256" windowHeight="12456" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="22932" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Users" sheetId="2" r:id="rId1"/>
@@ -170,7 +170,7 @@
     <t>FVATestOpportunity Admin</t>
   </si>
   <si>
-    <t>Bingo@123456</t>
+    <t>Bingo@12345</t>
   </si>
 </sst>
 </file>
@@ -815,10 +815,10 @@
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="B2" r:id="rId1" xr:uid="{00000000-0004-0000-0200-000000000000}"/>
-    <hyperlink ref="A2" r:id="rId2" xr:uid="{3445B329-E5DB-4611-B1CE-B0681D950C43}"/>
-    <hyperlink ref="A3" r:id="rId3" tooltip="mailto:klulla@hl.com.test" display="mailto:klulla@hl.com.test" xr:uid="{C8EC5463-FDDF-464D-9CB8-5D48135FBF68}"/>
-    <hyperlink ref="B3" r:id="rId4" xr:uid="{F66D924C-A8D1-422A-8461-D4309A4022A7}"/>
+    <hyperlink ref="A2" r:id="rId1" xr:uid="{3445B329-E5DB-4611-B1CE-B0681D950C43}"/>
+    <hyperlink ref="A3" r:id="rId2" tooltip="mailto:klulla@hl.com.test" display="mailto:klulla@hl.com.test" xr:uid="{C8EC5463-FDDF-464D-9CB8-5D48135FBF68}"/>
+    <hyperlink ref="B3" r:id="rId3" xr:uid="{F66D924C-A8D1-422A-8461-D4309A4022A7}"/>
+    <hyperlink ref="B2" r:id="rId4" xr:uid="{040B7D94-2E5B-42F8-A0F0-87295F1696DE}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -862,7 +862,7 @@
     <hyperlink ref="A2" r:id="rId1" tooltip="mailto:kspero@hl.com.test" display="mailto:kspero@hl.com.test" xr:uid="{BF9A316F-3890-4091-A712-BAB45FA8B7A3}"/>
     <hyperlink ref="A3" r:id="rId2" tooltip="mailto:klulla@hl.com.test" display="mailto:klulla@hl.com.test" xr:uid="{102C98B0-E08F-485E-82F8-4D662884A9CD}"/>
     <hyperlink ref="B2" r:id="rId3" xr:uid="{1E1DF281-9C0E-478E-A031-394BCFAD2AF4}"/>
-    <hyperlink ref="B3" r:id="rId4" xr:uid="{F1A2ACD0-B05E-48F1-B729-9A8B2F996DA6}"/>
+    <hyperlink ref="B3" r:id="rId4" xr:uid="{A5CB5B42-29B5-4C5E-92DF-57B2FE012305}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>